<commit_message>
Keep black console window intact after admin restart server
</commit_message>
<xml_diff>
--- a/publish/Math/questions.xlsx
+++ b/publish/Math/questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\anuj\opnsrc_try\ai\QuizWeb_Manual\publish\Math\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ACD56C4-72D4-454C-9794-93B5EED0522B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ACF7096-AF92-4BD4-BE6C-87E572F3B81F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
   <si>
     <t>Class: 9</t>
   </si>
@@ -73,217 +73,52 @@
     <t/>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
     <t>D</t>
   </si>
   <si>
     <t>E</t>
   </si>
   <si>
-    <t>Google Search</t>
-  </si>
-  <si>
-    <t>Google Drive</t>
-  </si>
-  <si>
-    <t>Google Chrome</t>
-  </si>
-  <si>
-    <t>Google Maps</t>
-  </si>
-  <si>
-    <t>Notepad</t>
-  </si>
-  <si>
-    <t>AnyDesk</t>
-  </si>
-  <si>
-    <t>Calculator</t>
-  </si>
-  <si>
-    <t>Paint</t>
-  </si>
-  <si>
-    <t>73</t>
-  </si>
-  <si>
-    <t>Which of the following is a video conferencing tool?</t>
-  </si>
-  <si>
-    <t>Google Meet</t>
-  </si>
-  <si>
-    <t>74</t>
-  </si>
-  <si>
-    <t>Zoom and Microsoft Teams are commonly used for:</t>
-  </si>
-  <si>
-    <t>Designing graphics</t>
-  </si>
-  <si>
-    <t>Compiling programs</t>
-  </si>
-  <si>
-    <t>Storing files</t>
-  </si>
-  <si>
-    <t>Video conferencing and online meetings</t>
-  </si>
-  <si>
-    <t>Browsing the web</t>
-  </si>
-  <si>
-    <t>75</t>
-  </si>
-  <si>
-    <t>In an online meeting, the "Mute" button is used to:</t>
-  </si>
-  <si>
-    <t>Turn off your camera</t>
-  </si>
-  <si>
-    <t>End the meeting</t>
-  </si>
-  <si>
-    <t>Share the screen</t>
-  </si>
-  <si>
-    <t>Record the meeting</t>
-  </si>
-  <si>
-    <t>Turn off your microphone</t>
-  </si>
-  <si>
-    <t>76</t>
-  </si>
-  <si>
-    <t>Remote desktop software allows a person to:</t>
-  </si>
-  <si>
-    <t>Access and control another computer over the Internet</t>
-  </si>
-  <si>
-    <t>Print documents on a network</t>
-  </si>
-  <si>
-    <t>Play CD-ROMs</t>
-  </si>
-  <si>
-    <t>Defragment the hard disk</t>
-  </si>
-  <si>
-    <t>Install drivers</t>
-  </si>
-  <si>
-    <t>77</t>
-  </si>
-  <si>
-    <t>Which of the following is NOT a remote access tool?</t>
-  </si>
-  <si>
-    <t>TeamViewer</t>
-  </si>
-  <si>
-    <t>Chrome Remote Desktop</t>
-  </si>
-  <si>
-    <t>AnyDesk Remote</t>
-  </si>
-  <si>
-    <t>78</t>
-  </si>
-  <si>
-    <t>Which tool is often used for screen sharing during an online class?</t>
-  </si>
-  <si>
-    <t>Zoom</t>
-  </si>
-  <si>
-    <t>Word Processor</t>
-  </si>
-  <si>
-    <t>79</t>
-  </si>
-  <si>
-    <t>Remote access between two computers generally requires:</t>
-  </si>
-  <si>
-    <t>A printer</t>
-  </si>
-  <si>
-    <t>A scanner</t>
-  </si>
-  <si>
-    <t>A projector</t>
-  </si>
-  <si>
-    <t>An Internet connection between both computers</t>
-  </si>
-  <si>
-    <t>A television</t>
-  </si>
-  <si>
-    <t>80</t>
-  </si>
-  <si>
-    <t>Which of the following is NOT a video conferencing application?</t>
-  </si>
-  <si>
-    <t>Microsoft Teams</t>
-  </si>
-  <si>
-    <t>Skype</t>
-  </si>
-  <si>
-    <t>81</t>
-  </si>
-  <si>
-    <t>UI stands for:</t>
-  </si>
-  <si>
-    <t>User Interface</t>
-  </si>
-  <si>
-    <t>User Internet</t>
-  </si>
-  <si>
-    <t>Universal Interface</t>
-  </si>
-  <si>
-    <t>User Input</t>
-  </si>
-  <si>
-    <t>Under Interface</t>
-  </si>
-  <si>
-    <t>82</t>
-  </si>
-  <si>
-    <t>UX stands for:</t>
-  </si>
-  <si>
-    <t>User External</t>
-  </si>
-  <si>
-    <t>User Experience</t>
-  </si>
-  <si>
-    <t>Universal Experience</t>
-  </si>
-  <si>
-    <t>User Expression</t>
-  </si>
-  <si>
-    <t>Unified Extension</t>
+    <t>css</t>
+  </si>
+  <si>
+    <t>www</t>
+  </si>
+  <si>
+    <t>109</t>
+  </si>
+  <si>
+    <t>Which of the following is a top-level domain?</t>
+  </si>
+  <si>
+    <t>http</t>
+  </si>
+  <si>
+    <t>html</t>
+  </si>
+  <si>
+    <t>.com</t>
+  </si>
+  <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>An ordered list in HTML displays items with:</t>
+  </si>
+  <si>
+    <t>Circles</t>
+  </si>
+  <si>
+    <t>Squares</t>
+  </si>
+  <si>
+    <t>Dashes</t>
+  </si>
+  <si>
+    <t>Check marks</t>
+  </si>
+  <si>
+    <t>Numbers</t>
   </si>
 </sst>
 </file>
@@ -1124,7 +959,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.4">
@@ -1185,292 +1020,66 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>22</v>
+      </c>
+      <c r="D5" t="s">
+        <v>16</v>
       </c>
       <c r="E5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H5" t="s">
+        <v>24</v>
+      </c>
+      <c r="I5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J5" t="s">
         <v>19</v>
-      </c>
-      <c r="F5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" t="s">
-        <v>32</v>
-      </c>
-      <c r="I5" t="s">
-        <v>23</v>
-      </c>
-      <c r="J5" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>34</v>
+        <v>27</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
       </c>
       <c r="E6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F6" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="G6" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="H6" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="I6" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="J6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" t="s">
-        <v>41</v>
-      </c>
-      <c r="E7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H7" t="s">
-        <v>44</v>
-      </c>
-      <c r="I7" t="s">
-        <v>45</v>
-      </c>
-      <c r="J7" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" t="s">
-        <v>48</v>
-      </c>
-      <c r="E8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" t="s">
-        <v>50</v>
-      </c>
-      <c r="H8" t="s">
-        <v>51</v>
-      </c>
-      <c r="I8" t="s">
-        <v>52</v>
-      </c>
-      <c r="J8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" t="s">
-        <v>29</v>
-      </c>
-      <c r="H9" t="s">
-        <v>56</v>
-      </c>
-      <c r="I9" t="s">
-        <v>57</v>
-      </c>
-      <c r="J9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G10" t="s">
-        <v>28</v>
-      </c>
-      <c r="H10" t="s">
-        <v>61</v>
-      </c>
-      <c r="I10" t="s">
-        <v>29</v>
-      </c>
-      <c r="J10" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>63</v>
-      </c>
-      <c r="B11" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" t="s">
-        <v>64</v>
-      </c>
-      <c r="E11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F11" t="s">
-        <v>65</v>
-      </c>
-      <c r="G11" t="s">
-        <v>66</v>
-      </c>
-      <c r="H11" t="s">
-        <v>67</v>
-      </c>
-      <c r="I11" t="s">
-        <v>68</v>
-      </c>
-      <c r="J11" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
-        <v>70</v>
-      </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" t="s">
-        <v>71</v>
-      </c>
-      <c r="E12" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" t="s">
         <v>32</v>
-      </c>
-      <c r="G12" t="s">
-        <v>61</v>
-      </c>
-      <c r="H12" t="s">
-        <v>72</v>
-      </c>
-      <c r="I12" t="s">
-        <v>73</v>
-      </c>
-      <c r="J12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>74</v>
-      </c>
-      <c r="B13" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" t="s">
-        <v>75</v>
-      </c>
-      <c r="E13" t="s">
-        <v>17</v>
-      </c>
-      <c r="F13" t="s">
-        <v>76</v>
-      </c>
-      <c r="G13" t="s">
-        <v>77</v>
-      </c>
-      <c r="H13" t="s">
-        <v>78</v>
-      </c>
-      <c r="I13" t="s">
-        <v>79</v>
-      </c>
-      <c r="J13" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
-        <v>81</v>
-      </c>
-      <c r="B14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" t="s">
-        <v>82</v>
-      </c>
-      <c r="E14" t="s">
-        <v>18</v>
-      </c>
-      <c r="F14" t="s">
-        <v>83</v>
-      </c>
-      <c r="G14" t="s">
-        <v>84</v>
-      </c>
-      <c r="H14" t="s">
-        <v>85</v>
-      </c>
-      <c r="I14" t="s">
-        <v>86</v>
-      </c>
-      <c r="J14" t="s">
-        <v>87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>